<commit_message>
Can create cells! But cif2cell does not give a complete conventional cell :(
</commit_message>
<xml_diff>
--- a/Timeliste.xlsx
+++ b/Timeliste.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erlen\Documents\Github\Crystallographic-Reality\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6C5E5A2-5F04-4CE7-A519-0C9D9E5632B5}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62596F05-A73C-4B06-8D94-D3072DC18A38}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{36930395-203A-46D0-A2AB-0BDFDA6E0730}"/>
   </bookViews>
@@ -440,7 +440,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
@@ -489,6 +489,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="4" fillId="2" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -837,7 +838,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{452BBFAB-770E-4EEE-86BF-79330E4925BB}">
-  <dimension ref="A1:K35"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.7109375" bestFit="1" customWidth="1"/>
@@ -849,14 +850,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="27" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="30"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="31"/>
     </row>
     <row r="2" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -888,25 +889,25 @@
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="31" t="s">
+      <c r="B5" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="31"/>
-      <c r="D5" s="31"/>
-      <c r="E5" s="31"/>
-      <c r="F5" s="32"/>
+      <c r="C5" s="32"/>
+      <c r="D5" s="32"/>
+      <c r="E5" s="32"/>
+      <c r="F5" s="33"/>
     </row>
     <row r="6" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="31" t="s">
+      <c r="B6" s="32" t="s">
         <v>24</v>
       </c>
-      <c r="C6" s="31"/>
-      <c r="D6" s="31"/>
-      <c r="E6" s="31"/>
-      <c r="F6" s="32"/>
+      <c r="C6" s="32"/>
+      <c r="D6" s="32"/>
+      <c r="E6" s="32"/>
+      <c r="F6" s="33"/>
     </row>
     <row r="7" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
@@ -1076,7 +1077,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A17" s="5">
         <v>44369</v>
       </c>
@@ -1098,7 +1099,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A18" s="5">
         <v>44382</v>
       </c>
@@ -1106,35 +1107,41 @@
         <v>0.55069444444444449</v>
       </c>
       <c r="C18" s="6">
-        <v>0.69652777777777775</v>
+        <v>0.70694444444444438</v>
       </c>
       <c r="D18" s="7">
         <f t="shared" si="0"/>
-        <v>0.14583333333333326</v>
+        <v>0.15624999999999989</v>
       </c>
       <c r="E18" s="8">
         <f t="shared" si="1"/>
-        <v>3.4999999999999982</v>
+        <v>3.7499999999999973</v>
       </c>
       <c r="F18" s="9" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A19" s="10"/>
-      <c r="B19" s="6"/>
-      <c r="C19" s="6"/>
-      <c r="D19" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E19" s="8" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
+    <row r="19" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A19" s="5">
+        <v>44383</v>
+      </c>
+      <c r="B19" s="6">
+        <v>0.5625</v>
+      </c>
+      <c r="C19" s="6">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="D19" s="7">
+        <f t="shared" si="0"/>
+        <v>0.10416666666666663</v>
+      </c>
+      <c r="E19" s="8">
+        <f t="shared" si="1"/>
+        <v>2.4999999999999991</v>
       </c>
       <c r="F19" s="9"/>
     </row>
-    <row r="20" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A20" s="10"/>
       <c r="B20" s="6"/>
       <c r="C20" s="6"/>
@@ -1148,7 +1155,7 @@
       </c>
       <c r="F20" s="9"/>
     </row>
-    <row r="21" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A21" s="10"/>
       <c r="B21" s="6"/>
       <c r="C21" s="6"/>
@@ -1162,7 +1169,7 @@
       </c>
       <c r="F21" s="9"/>
     </row>
-    <row r="22" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A22" s="10"/>
       <c r="B22" s="6"/>
       <c r="C22" s="6"/>
@@ -1176,7 +1183,7 @@
       </c>
       <c r="F22" s="9"/>
     </row>
-    <row r="23" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A23" s="10"/>
       <c r="B23" s="6"/>
       <c r="C23" s="6"/>
@@ -1190,7 +1197,7 @@
       </c>
       <c r="F23" s="9"/>
     </row>
-    <row r="24" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A24" s="10"/>
       <c r="B24" s="6"/>
       <c r="C24" s="6"/>
@@ -1204,7 +1211,7 @@
       </c>
       <c r="F24" s="9"/>
     </row>
-    <row r="25" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A25" s="10"/>
       <c r="B25" s="6"/>
       <c r="C25" s="6"/>
@@ -1218,7 +1225,7 @@
       </c>
       <c r="F25" s="9"/>
     </row>
-    <row r="26" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A26" s="10"/>
       <c r="B26" s="6"/>
       <c r="C26" s="6"/>
@@ -1231,12 +1238,8 @@
         <v xml:space="preserve"> </v>
       </c>
       <c r="F26" s="9"/>
-      <c r="K26">
-        <f>120-17.5</f>
-        <v>102.5</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="27" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A27" s="10"/>
       <c r="B27" s="6"/>
       <c r="C27" s="6"/>
@@ -1250,7 +1253,7 @@
       </c>
       <c r="F27" s="9"/>
     </row>
-    <row r="28" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A28" s="10"/>
       <c r="B28" s="6"/>
       <c r="C28" s="6"/>
@@ -1264,7 +1267,7 @@
       </c>
       <c r="F28" s="9"/>
     </row>
-    <row r="29" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A29" s="10"/>
       <c r="B29" s="6"/>
       <c r="C29" s="6"/>
@@ -1278,7 +1281,7 @@
       </c>
       <c r="F29" s="9"/>
     </row>
-    <row r="30" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A30" s="10"/>
       <c r="B30" s="6"/>
       <c r="C30" s="6"/>
@@ -1292,7 +1295,7 @@
       </c>
       <c r="F30" s="9"/>
     </row>
-    <row r="31" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A31" s="10"/>
       <c r="B31" s="6"/>
       <c r="C31" s="6"/>
@@ -1306,7 +1309,7 @@
       </c>
       <c r="F31" s="9"/>
     </row>
-    <row r="32" spans="1:11" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:6" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="10"/>
       <c r="B32" s="6"/>
       <c r="C32" s="6"/>
@@ -1320,19 +1323,19 @@
       </c>
       <c r="F32" s="12"/>
     </row>
-    <row r="33" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A33" s="13"/>
       <c r="B33" s="14"/>
       <c r="C33" s="15"/>
       <c r="D33" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="E33" s="33" t="s">
+      <c r="E33" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="F33" s="34"/>
-    </row>
-    <row r="34" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="F33" s="35"/>
+    </row>
+    <row r="34" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A34" s="17"/>
       <c r="B34" s="15"/>
       <c r="C34" s="3" t="s">
@@ -1340,12 +1343,16 @@
       </c>
       <c r="D34" s="18">
         <f>SUM(D12:D32)</f>
-        <v>0.87499999999999989</v>
-      </c>
-      <c r="E34" s="35"/>
-      <c r="F34" s="36"/>
-    </row>
-    <row r="35" spans="1:6" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+        <v>0.98958333333333315</v>
+      </c>
+      <c r="E34" s="36"/>
+      <c r="F34" s="37"/>
+      <c r="H34" s="28">
+        <f>120-D35</f>
+        <v>96.25</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="19"/>
       <c r="B35" s="20"/>
       <c r="C35" s="21" t="s">
@@ -1353,10 +1360,10 @@
       </c>
       <c r="D35" s="22">
         <f>SUM(E12:E32)</f>
-        <v>21</v>
-      </c>
-      <c r="E35" s="37"/>
-      <c r="F35" s="38"/>
+        <v>23.749999999999996</v>
+      </c>
+      <c r="E35" s="38"/>
+      <c r="F35" s="39"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
.xyz-file does not give cell length as expected
</commit_message>
<xml_diff>
--- a/Timeliste.xlsx
+++ b/Timeliste.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erlen\Documents\Github\Crystallographic-Reality\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62596F05-A73C-4B06-8D94-D3072DC18A38}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0FB1361-5DDD-4EC2-9414-984A758147CE}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{36930395-203A-46D0-A2AB-0BDFDA6E0730}"/>
   </bookViews>
@@ -1142,16 +1142,22 @@
       <c r="F19" s="9"/>
     </row>
     <row r="20" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A20" s="10"/>
-      <c r="B20" s="6"/>
-      <c r="C20" s="6"/>
-      <c r="D20" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E20" s="8" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
+      <c r="A20" s="5">
+        <v>44383</v>
+      </c>
+      <c r="B20" s="6">
+        <v>0.6875</v>
+      </c>
+      <c r="C20" s="6">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="D20" s="7">
+        <f t="shared" si="0"/>
+        <v>0.10416666666666663</v>
+      </c>
+      <c r="E20" s="8">
+        <f t="shared" si="1"/>
+        <v>2.4999999999999991</v>
       </c>
       <c r="F20" s="9"/>
     </row>
@@ -1343,13 +1349,13 @@
       </c>
       <c r="D34" s="18">
         <f>SUM(D12:D32)</f>
-        <v>0.98958333333333315</v>
+        <v>1.0937499999999998</v>
       </c>
       <c r="E34" s="36"/>
       <c r="F34" s="37"/>
       <c r="H34" s="28">
         <f>120-D35</f>
-        <v>96.25</v>
+        <v>93.75</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -1360,7 +1366,7 @@
       </c>
       <c r="D35" s="22">
         <f>SUM(E12:E32)</f>
-        <v>23.749999999999996</v>
+        <v>26.249999999999996</v>
       </c>
       <c r="E35" s="38"/>
       <c r="F35" s="39"/>

</xml_diff>

<commit_message>
Fixed cell generation for corners, sides, and edges
</commit_message>
<xml_diff>
--- a/Timeliste.xlsx
+++ b/Timeliste.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erlen\Documents\Github\Crystallographic-Reality\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0FB1361-5DDD-4EC2-9414-984A758147CE}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71511F2D-12B2-4380-8935-908067C00D69}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{36930395-203A-46D0-A2AB-0BDFDA6E0730}"/>
   </bookViews>
@@ -1162,16 +1162,22 @@
       <c r="F20" s="9"/>
     </row>
     <row r="21" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A21" s="10"/>
-      <c r="B21" s="6"/>
-      <c r="C21" s="6"/>
-      <c r="D21" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E21" s="8" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
+      <c r="A21" s="5">
+        <v>44392</v>
+      </c>
+      <c r="B21" s="6">
+        <v>0.68402777777777779</v>
+      </c>
+      <c r="C21" s="6">
+        <v>0.88194444444444453</v>
+      </c>
+      <c r="D21" s="7">
+        <f t="shared" si="0"/>
+        <v>0.19791666666666674</v>
+      </c>
+      <c r="E21" s="8">
+        <f t="shared" si="1"/>
+        <v>4.7500000000000018</v>
       </c>
       <c r="F21" s="9"/>
     </row>
@@ -1349,13 +1355,13 @@
       </c>
       <c r="D34" s="18">
         <f>SUM(D12:D32)</f>
-        <v>1.0937499999999998</v>
+        <v>1.2916666666666665</v>
       </c>
       <c r="E34" s="36"/>
       <c r="F34" s="37"/>
       <c r="H34" s="28">
         <f>120-D35</f>
-        <v>93.75</v>
+        <v>89</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -1366,7 +1372,7 @@
       </c>
       <c r="D35" s="22">
         <f>SUM(E12:E32)</f>
-        <v>26.249999999999996</v>
+        <v>31</v>
       </c>
       <c r="E35" s="38"/>
       <c r="F35" s="39"/>

</xml_diff>

<commit_message>
Tested some concepts, updated packages, made some plans going forward
</commit_message>
<xml_diff>
--- a/Timeliste.xlsx
+++ b/Timeliste.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erlen\Documents\Github\Crystallographic-Reality\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71511F2D-12B2-4380-8935-908067C00D69}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D956B93A-DEFF-4BFA-929C-52D0DD0A70D4}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{36930395-203A-46D0-A2AB-0BDFDA6E0730}"/>
   </bookViews>
@@ -1182,16 +1182,22 @@
       <c r="F21" s="9"/>
     </row>
     <row r="22" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A22" s="10"/>
-      <c r="B22" s="6"/>
-      <c r="C22" s="6"/>
-      <c r="D22" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E22" s="8" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
+      <c r="A22" s="5">
+        <v>44396</v>
+      </c>
+      <c r="B22" s="6">
+        <v>0.68055555555555547</v>
+      </c>
+      <c r="C22" s="6">
+        <v>0.77083333333333337</v>
+      </c>
+      <c r="D22" s="7">
+        <f t="shared" si="0"/>
+        <v>9.0277777777777901E-2</v>
+      </c>
+      <c r="E22" s="8">
+        <f t="shared" si="1"/>
+        <v>2.1666666666666696</v>
       </c>
       <c r="F22" s="9"/>
     </row>
@@ -1355,13 +1361,13 @@
       </c>
       <c r="D34" s="18">
         <f>SUM(D12:D32)</f>
-        <v>1.2916666666666665</v>
+        <v>1.3819444444444444</v>
       </c>
       <c r="E34" s="36"/>
       <c r="F34" s="37"/>
       <c r="H34" s="28">
         <f>120-D35</f>
-        <v>89</v>
+        <v>86.833333333333329</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -1372,7 +1378,7 @@
       </c>
       <c r="D35" s="22">
         <f>SUM(E12:E32)</f>
-        <v>31</v>
+        <v>33.166666666666671</v>
       </c>
       <c r="E35" s="38"/>
       <c r="F35" s="39"/>

</xml_diff>

<commit_message>
Added Unit Cell borders with functional angles
</commit_message>
<xml_diff>
--- a/Timeliste.xlsx
+++ b/Timeliste.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erlen\Documents\Github\Crystallographic-Reality\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D956B93A-DEFF-4BFA-929C-52D0DD0A70D4}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F282FAEB-2F62-44FE-82AF-C041BABFA3BD}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{36930395-203A-46D0-A2AB-0BDFDA6E0730}"/>
   </bookViews>
@@ -440,7 +440,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
@@ -490,6 +490,8 @@
     <xf numFmtId="49" fontId="4" fillId="2" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -850,14 +852,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="27" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="31"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="33"/>
     </row>
     <row r="2" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -889,25 +891,25 @@
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="32" t="s">
+      <c r="B5" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="32"/>
-      <c r="D5" s="32"/>
-      <c r="E5" s="32"/>
-      <c r="F5" s="33"/>
+      <c r="C5" s="34"/>
+      <c r="D5" s="34"/>
+      <c r="E5" s="34"/>
+      <c r="F5" s="35"/>
     </row>
     <row r="6" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="32" t="s">
+      <c r="B6" s="34" t="s">
         <v>24</v>
       </c>
-      <c r="C6" s="32"/>
-      <c r="D6" s="32"/>
-      <c r="E6" s="32"/>
-      <c r="F6" s="33"/>
+      <c r="C6" s="34"/>
+      <c r="D6" s="34"/>
+      <c r="E6" s="34"/>
+      <c r="F6" s="35"/>
     </row>
     <row r="7" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
@@ -1202,16 +1204,22 @@
       <c r="F22" s="9"/>
     </row>
     <row r="23" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A23" s="10"/>
-      <c r="B23" s="6"/>
-      <c r="C23" s="6"/>
-      <c r="D23" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E23" s="8" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
+      <c r="A23" s="5">
+        <v>44397</v>
+      </c>
+      <c r="B23" s="6">
+        <v>0.67361111111111116</v>
+      </c>
+      <c r="C23" s="6">
+        <v>0.85416666666666663</v>
+      </c>
+      <c r="D23" s="7">
+        <f t="shared" si="0"/>
+        <v>0.18055555555555547</v>
+      </c>
+      <c r="E23" s="8">
+        <f t="shared" si="1"/>
+        <v>4.3333333333333313</v>
       </c>
       <c r="F23" s="9"/>
     </row>
@@ -1348,10 +1356,11 @@
       <c r="D33" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="E33" s="34" t="s">
+      <c r="E33" s="36" t="s">
         <v>16</v>
       </c>
-      <c r="F33" s="35"/>
+      <c r="F33" s="37"/>
+      <c r="H33" s="30"/>
     </row>
     <row r="34" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A34" s="17"/>
@@ -1361,14 +1370,11 @@
       </c>
       <c r="D34" s="18">
         <f>SUM(D12:D32)</f>
-        <v>1.3819444444444444</v>
-      </c>
-      <c r="E34" s="36"/>
-      <c r="F34" s="37"/>
-      <c r="H34" s="28">
-        <f>120-D35</f>
-        <v>86.833333333333329</v>
-      </c>
+        <v>1.5625</v>
+      </c>
+      <c r="E34" s="38"/>
+      <c r="F34" s="39"/>
+      <c r="H34" s="29"/>
     </row>
     <row r="35" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="19"/>
@@ -1378,10 +1384,14 @@
       </c>
       <c r="D35" s="22">
         <f>SUM(E12:E32)</f>
-        <v>33.166666666666671</v>
-      </c>
-      <c r="E35" s="38"/>
-      <c r="F35" s="39"/>
+        <v>37.5</v>
+      </c>
+      <c r="E35" s="40"/>
+      <c r="F35" s="41"/>
+      <c r="H35" s="28">
+        <f>120-D35</f>
+        <v>82.5</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
Re-did planes to work with for cellAngles not equal to 90 and coded cellVectors based on fractional coordinates
</commit_message>
<xml_diff>
--- a/Timeliste.xlsx
+++ b/Timeliste.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erlen\Documents\Github\Crystallographic-Reality\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5CBA0B2-F5DA-40E6-AB7D-B1BD4EA0AC47}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C27BAC7-73A5-4ABC-BE49-6085E6EF47D7}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{36930395-203A-46D0-A2AB-0BDFDA6E0730}"/>
+    <workbookView xWindow="5895" yWindow="3315" windowWidth="21600" windowHeight="11385" xr2:uid="{36930395-203A-46D0-A2AB-0BDFDA6E0730}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -1231,29 +1231,35 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="C24" s="6">
-        <v>0.90625</v>
+        <v>0.91666666666666663</v>
       </c>
       <c r="D24" s="7">
         <f t="shared" si="0"/>
-        <v>0.20833333333333337</v>
+        <v>0.21875</v>
       </c>
       <c r="E24" s="8">
         <f t="shared" si="1"/>
-        <v>5.0000000000000009</v>
+        <v>5.25</v>
       </c>
       <c r="F24" s="9"/>
     </row>
     <row r="25" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A25" s="10"/>
-      <c r="B25" s="6"/>
-      <c r="C25" s="6"/>
-      <c r="D25" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E25" s="8" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
+      <c r="A25" s="5">
+        <v>44400</v>
+      </c>
+      <c r="B25" s="6">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="C25" s="6">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="D25" s="7">
+        <f t="shared" si="0"/>
+        <v>0.20833333333333326</v>
+      </c>
+      <c r="E25" s="8">
+        <f t="shared" si="1"/>
+        <v>4.9999999999999982</v>
       </c>
       <c r="F25" s="9"/>
     </row>
@@ -1376,7 +1382,7 @@
       </c>
       <c r="D34" s="18">
         <f>SUM(D12:D32)</f>
-        <v>1.7708333333333335</v>
+        <v>1.9895833333333333</v>
       </c>
       <c r="E34" s="38"/>
       <c r="F34" s="39"/>
@@ -1390,13 +1396,13 @@
       </c>
       <c r="D35" s="22">
         <f>SUM(E12:E32)</f>
-        <v>42.5</v>
+        <v>47.75</v>
       </c>
       <c r="E35" s="40"/>
       <c r="F35" s="41"/>
       <c r="H35" s="28">
         <f>120-D35</f>
-        <v>77.5</v>
+        <v>72.25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Made CreatePlane() work for all planes in all axis directions.
Need to determine crystal system to set planes, axis etc. correctly according to the Hermann-Mauguin notation
</commit_message>
<xml_diff>
--- a/Timeliste.xlsx
+++ b/Timeliste.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23801"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erlen\Documents\Github\Crystallographic-Reality\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C27BAC7-73A5-4ABC-BE49-6085E6EF47D7}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{027C026F-D51F-4ED4-A5CD-840D41DA3FC3}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5895" yWindow="3315" windowWidth="21600" windowHeight="11385" xr2:uid="{36930395-203A-46D0-A2AB-0BDFDA6E0730}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{36930395-203A-46D0-A2AB-0BDFDA6E0730}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -1264,16 +1264,22 @@
       <c r="F25" s="9"/>
     </row>
     <row r="26" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A26" s="10"/>
-      <c r="B26" s="6"/>
-      <c r="C26" s="6"/>
-      <c r="D26" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E26" s="8" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
+      <c r="A26" s="5">
+        <v>44403</v>
+      </c>
+      <c r="B26" s="6">
+        <v>0.72569444444444453</v>
+      </c>
+      <c r="C26" s="6">
+        <v>0.84027777777777779</v>
+      </c>
+      <c r="D26" s="7">
+        <f t="shared" si="0"/>
+        <v>0.11458333333333326</v>
+      </c>
+      <c r="E26" s="8">
+        <f t="shared" si="1"/>
+        <v>2.7499999999999982</v>
       </c>
       <c r="F26" s="9"/>
     </row>
@@ -1382,7 +1388,7 @@
       </c>
       <c r="D34" s="18">
         <f>SUM(D12:D32)</f>
-        <v>1.9895833333333333</v>
+        <v>2.1041666666666665</v>
       </c>
       <c r="E34" s="38"/>
       <c r="F34" s="39"/>
@@ -1396,13 +1402,13 @@
       </c>
       <c r="D35" s="22">
         <f>SUM(E12:E32)</f>
-        <v>47.75</v>
+        <v>50.5</v>
       </c>
       <c r="E35" s="40"/>
       <c r="F35" s="41"/>
       <c r="H35" s="28">
         <f>120-D35</f>
-        <v>72.25</v>
+        <v>69.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Planned ahead for generating symmetries.
See README.md for proposed algorithm for converting from matrix to visual symmetry operation
</commit_message>
<xml_diff>
--- a/Timeliste.xlsx
+++ b/Timeliste.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erlen\Documents\Github\Crystallographic-Reality\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{027C026F-D51F-4ED4-A5CD-840D41DA3FC3}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{799E6DD7-5E1D-4339-90BD-02309ADBA622}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{36930395-203A-46D0-A2AB-0BDFDA6E0730}"/>
   </bookViews>
@@ -1284,16 +1284,22 @@
       <c r="F26" s="9"/>
     </row>
     <row r="27" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A27" s="10"/>
-      <c r="B27" s="6"/>
-      <c r="C27" s="6"/>
-      <c r="D27" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E27" s="8" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
+      <c r="A27" s="5">
+        <v>44404</v>
+      </c>
+      <c r="B27" s="6">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="C27" s="6">
+        <v>0.77083333333333337</v>
+      </c>
+      <c r="D27" s="7">
+        <f t="shared" si="0"/>
+        <v>0.10416666666666674</v>
+      </c>
+      <c r="E27" s="8">
+        <f t="shared" si="1"/>
+        <v>2.5000000000000018</v>
       </c>
       <c r="F27" s="9"/>
     </row>
@@ -1388,7 +1394,7 @@
       </c>
       <c r="D34" s="18">
         <f>SUM(D12:D32)</f>
-        <v>2.1041666666666665</v>
+        <v>2.208333333333333</v>
       </c>
       <c r="E34" s="38"/>
       <c r="F34" s="39"/>
@@ -1402,13 +1408,13 @@
       </c>
       <c r="D35" s="22">
         <f>SUM(E12:E32)</f>
-        <v>50.5</v>
+        <v>53</v>
       </c>
       <c r="E35" s="40"/>
       <c r="F35" s="41"/>
       <c r="H35" s="28">
         <f>120-D35</f>
-        <v>69.5</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implemented UI-menu to select .cif-file, fixed minor bugs, and had "fun" with cif2cell
</commit_message>
<xml_diff>
--- a/Timeliste.xlsx
+++ b/Timeliste.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erlen\Documents\Github\Crystallographic-Reality\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{799E6DD7-5E1D-4339-90BD-02309ADBA622}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE2EA56C-E363-4CD7-AB26-E0E8E11E084A}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{36930395-203A-46D0-A2AB-0BDFDA6E0730}"/>
   </bookViews>
@@ -1304,16 +1304,22 @@
       <c r="F27" s="9"/>
     </row>
     <row r="28" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A28" s="10"/>
-      <c r="B28" s="6"/>
-      <c r="C28" s="6"/>
-      <c r="D28" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E28" s="8" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
+      <c r="A28" s="5">
+        <v>44406</v>
+      </c>
+      <c r="B28" s="6">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="C28" s="6">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="D28" s="7">
+        <f t="shared" si="0"/>
+        <v>0.25</v>
+      </c>
+      <c r="E28" s="8">
+        <f t="shared" si="1"/>
+        <v>6</v>
       </c>
       <c r="F28" s="9"/>
     </row>
@@ -1394,7 +1400,7 @@
       </c>
       <c r="D34" s="18">
         <f>SUM(D12:D32)</f>
-        <v>2.208333333333333</v>
+        <v>2.458333333333333</v>
       </c>
       <c r="E34" s="38"/>
       <c r="F34" s="39"/>
@@ -1408,13 +1414,13 @@
       </c>
       <c r="D35" s="22">
         <f>SUM(E12:E32)</f>
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="E35" s="40"/>
       <c r="F35" s="41"/>
       <c r="H35" s="28">
         <f>120-D35</f>
-        <v>67</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>